<commit_message>
feat(geocoding): parse all 9 workbook sheets (Armazéns, Frota, Regras, Rotas, Motoristas) automatically upon upload in Georreferenciação
</commit_message>
<xml_diff>
--- a/Ficheiros EXCEL/PedroLopes/GeoRoute_Completo_Teste_2026-08-31.xlsx
+++ b/Ficheiros EXCEL/PedroLopes/GeoRoute_Completo_Teste_2026-08-31.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo\.gemini\antigravity\playground\core-omega\PRJT_GEO\Ficheiros EXCEL\PedroLopes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76B969B-9BB8-453B-81C1-DC318FE057C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{970EACA7-2B34-44F6-B73F-88E3F431E1F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="525" yWindow="-15855" windowWidth="27465" windowHeight="15135" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12806" uniqueCount="2394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12782" uniqueCount="2394">
   <si>
     <t>Nome_Armazem</t>
   </si>
@@ -38773,99 +38773,51 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>2033</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
       <c r="D2" s="4"/>
     </row>
     <row r="3" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>2033</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>42</v>
-      </c>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
       <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>2033</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>43</v>
-      </c>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
       <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>2033</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>44</v>
-      </c>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
       <c r="D5" s="7"/>
     </row>
     <row r="6" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>2033</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>45</v>
-      </c>
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
       <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>2033</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>46</v>
-      </c>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
       <c r="D7" s="7"/>
     </row>
     <row r="8" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>2033</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>47</v>
-      </c>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
       <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>2033</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>48</v>
-      </c>
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
       <c r="D9" s="7"/>
     </row>
   </sheetData>

</xml_diff>